<commit_message>
Add missing Config key LogMessage_GetTransactionData
</commit_message>
<xml_diff>
--- a/Job_Scraping_Project/Data/Config.xlsx
+++ b/Job_Scraping_Project/Data/Config.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -484,7 +484,6 @@
           <t>OrchestratorQueueName</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -492,7 +491,6 @@
           <t>OrchestratorQueueFolder</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -551,6 +549,18 @@
       <c r="B12" t="inlineStr">
         <is>
           <t xml:space="preserve">Error getting transaction data at transaction number: </t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>LogMessage_GetTransactionData</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New transaction retrieved: </t>
         </is>
       </c>
     </row>

</xml_diff>